<commit_message>
Atualização automática da planilha via Apps Script
</commit_message>
<xml_diff>
--- a/Controle_Lote_Validade.xlsx
+++ b/Controle_Lote_Validade.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="1212">
-  <si>
-    <t>SKU</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="1211">
+  <si>
+    <t>Código do Produto</t>
   </si>
   <si>
     <t>Descrição</t>
@@ -3641,9 +3641,6 @@
   </si>
   <si>
     <t>Código item</t>
-  </si>
-  <si>
-    <t>Código do Produto</t>
   </si>
   <si>
     <t xml:space="preserve">KIT SABONETE VEGETAL HIDRATANTE TERRA DO SOL	3 UN 80G		</t>
@@ -14065,7 +14062,7 @@
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="35" t="s">
-        <v>1209</v>
+        <v>0</v>
       </c>
       <c r="D1" s="36" t="s">
         <v>1</v>
@@ -14525,7 +14522,7 @@
         <v>509</v>
       </c>
       <c r="D24" s="39" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="E24" s="41" t="str">
         <f t="array" ref="E24">XLOOKUP($A24,Lotes!$A:$A,Lotes!$C:$C)</f>
@@ -14645,7 +14642,7 @@
         <v>481</v>
       </c>
       <c r="D30" s="44" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="E30" s="41" t="str">
         <f t="array" ref="E30">XLOOKUP($A30,Lotes!$A:$A,Lotes!$C:$C)</f>

</xml_diff>